<commit_message>
M1 SKU: replace non-chemistry names; M2 March reference: add Методология sheet
M1 weekly_report.xlsx:
- ABC-KIT-018: «Набор кастрюль премиум 5 предметов» → «Универсальный обезжириватель кухни 750мл»
- ABC-KIT-031: «Сковорода керамическая 28см» → «Чистящее средство для духовки и плиты 500мл»
- ABC-GLS-012: «Набор бокалов универсал 6шт» → «Средство для мытья окон и зеркал 750мл»
- Highlights обновлён под новое название GLS-012
- Цифры (выручка, WoW, статус) не меняются

pnl-2026-03.xlsx:
- + лист «Методология» с явной базой расчёта по каждой статье:
  Комиссия от чистой, ДРР от валовой, Соинвест от net Ozon (refund сторнирует),
  Себестоимость = qty × weighted avg ₽/шт, и т.д.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pnl-2026-03.xlsx
+++ b/pnl-2026-03.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Источники" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Валовая" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Маржинальная" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Постоянные" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Операционная" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Свод" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Методология" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Источники" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Валовая" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Маржинальная" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Постоянные" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Операционная" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Свод" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -53,8 +54,16 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -67,14 +76,34 @@
         <bgColor rgb="FF666699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00305496"/>
+        <bgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="6">
@@ -87,7 +116,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -103,6 +132,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -353,6 +389,256 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="4" min="1" max="1"/>
+    <col width="72" customWidth="1" style="4" min="2" max="2"/>
+    <col width="50" customWidth="1" style="4" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="4">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Методология расчёта статей P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" s="4">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>База расчёта</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1" s="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Чистая выручка</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Валовая выручка − Возвраты по этой строке</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Источники (G = E − F)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1" s="4">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Себестоимость</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>qty проданных (только refund=N) × средневзвешенная ₽/шт по SKU</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>1c-production.xlsx → Σ(qty × cost_pu)/Σ(qty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1" s="4">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Комиссия</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Чистая выручка строки × Комиссия % канала</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>tariffs.xlsx → Комиссия, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1" s="4">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Логистика</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>qty (только refund=N) × Логистика ₽/шт канала</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>tariffs.xlsx → Логистика, ₽/шт</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1" s="4">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Эквайринг</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Включён в комиссию маркетплейса (отдельно не выделяется)</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1" s="4">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>ДРР (реклама)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Валовая выручка строки × ДРР % канала. ВАЖНО: база — валовая, не чистая</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>tariffs.xlsx → ДРР, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1" s="4">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Соинвест Озон</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Чистая выручка Озон-строки × % периода по SKU. Знак qty учитывается: refund=Y → соинвест сторнируется (отрицательный). WB соинвеста нет.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>ozon-coinvest.xlsx → % баллов по периоду и SKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1" s="4">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Маржинальная прибыль</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Валовая прибыль − Комиссия − Логистика − Эквайринг − ДРР + Соинвест (см. формулу на листе «Маржинальная»)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Маржинальная (J = D − E − F − G − H + I)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1" s="4">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Постоянные</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Σ 5 статей opex (ФОТ, Аренда, IT, Прочие услуги, Прочие административные). Аллокация по категориям пропорционально доле выручки.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>opex.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1" s="4">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Бренд-маркетинг</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Пул бренд-рекламы (отдельная строка ниже маржинальной). Аллокация по категориям пропорционально доле выручки.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>opex.xlsx → Бренд-реклама</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1" s="4">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Транспорт завод→FBO</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Пул транспортных расходов (отдельная строка ниже маржинальной). Аллокация по категориям пропорционально доле выручки.</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>opex.xlsx → Транспорт завод→FBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1" s="4">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Маржинальная − Постоянные − Бренд − Транспорт (по категориям и в сумме)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Операционная (H = C − E − F − G)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -1008,7 +1294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1374,7 +1660,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1952,7 +2238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2045,7 +2331,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2273,7 +2559,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
pnl-2026-03 Методология: strengthen ДРР row — emphasize «in margin, not opex»
Чтобы Claude не пропускал колонку tariffs.ДРР_% при сборке апрельского/майского P&L.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pnl-2026-03.xlsx
+++ b/pnl-2026-03.xlsx
@@ -408,6 +408,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="4">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -518,12 +519,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Валовая выручка строки × ДРР % канала. ВАЖНО: база — валовая, не чистая</t>
+          <t>Валовая выручка строки × ДРР % канала. ВАЖНО: ДРР учитывается в МАРЖИНАЛЬНОЙ (per-row, минус), а НЕ в opex. База — валовая выручка, не чистая.</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>tariffs.xlsx → ДРР, %</t>
+          <t>tariffs.xlsx → колонка «ДРР, %»</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pnl-2026-03 Источники: add column-header comments explaining each calculation
10 hover-комментариев к заголовкам колонок (Объём, Валовая, Возврат, Чистая,
Себестоимость, Комиссия, Логистика, Эквайринг, ДРР, Соинвест) — явно
прописывают базу расчёта и источник %.

Чтобы Claude не пропускал колонку tariffs.ДРР_% и не путал базы (комиссия
от чистой, ДРР от валовой) при сборке апрельского/майского P&L.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pnl-2026-03.xlsx
+++ b/pnl-2026-03.xlsx
@@ -212,6 +212,66 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Курс gls-ai-agents</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>qty проданных за период (только Refund=N, без возвратов).</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>qty × цена реализации. Только Refund=N. Возвраты — отдельной строкой.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Сумма возвратов = qty(Refund=Y) × цена. Хранится как положительное число, потом вычитается из Валовой.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>= Валовая − Возврат. Это база для Комиссии и Соинвеста.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>= qty(Refund=N) × weighted_avg ₽/шт SKU. weighted_avg = Σ(qty × cost_pu)/Σ(qty) по партиям. Источник: 1c-production.xlsx.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>= Чистая выручка × Комиссия_% канала. Источник %: tariffs.xlsx → колонка «Комиссия, %».</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>= qty(Refund=N) × Логистика_₽/шт канала. Источник: tariffs.xlsx → колонка «Логистика, ₽/шт».</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Включён в комиссию маркетплейса. Отдельно не выделяется (= 0 в этой таблице).</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>= ВАЛОВАЯ выручка × ДРР_% канала. ВАЖНО: база — валовая, не чистая. Источник %: tariffs.xlsx → колонка «ДРР, %». ДРР учитывается в МАРЖИНАЛЬНОЙ (минус), а НЕ в opex.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>= qty × цена × % периода (для Ozon-строк). qty со знаком: Refund=Y → отрицательный соинвест (сторно). WB соинвеста нет. Источник %: ozon-coinvest.xlsx. Знак в маржинальной — ПЛЮС (доход от Ozon).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -408,7 +468,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="4">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1292,6 +1351,7 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>